<commit_message>
docs: finalize v1.1.0 documentation and synchronize Korean guides
- Align English and Korean READMEs, ticket specifications, and design docs
  with the completed portfolio scope and current implementation
- Document verified resolved-ticket auto-close and hourly Supabase Cron
  execution, including the 168-hour eligibility rule
- Add bilingual auto-close scheduling decision logs and register them
  in the document catalog with localized titles and descriptions
- Clarify work-session permissions, approval force apply, and manual
  assignment and recipient validation limitations
- Update architecture terminology, examples, and reference workbooks,
  including NOTE authorization and auto-close rules
- Preserve historical decisions, deferred production scope, and known
  Storybook verification limitations
</commit_message>
<xml_diff>
--- a/docs/en/03-domain/service-desk/ticket/reference/restrict-employee-list.xlsx
+++ b/docs/en/03-domain/service-desk/ticket/reference/restrict-employee-list.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1182" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1182" uniqueCount="229">
   <si>
     <t>Service Desk Employee Reference Scope Matrix</t>
   </si>
@@ -696,6 +696,48 @@
   </si>
   <si>
     <t>Repository code and current design evidence answer the recorded question.</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/forms/ticket-form.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/forms/ticket-form.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/ui/dashboard-and-insight.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/ui/dashboard-and-insight.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/ui/dashboard-and-insight.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/ui/dashboard-and-insight.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/forms/ticket-form.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/forms/ticket-form.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/ui/dashboard-and-insight.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/ui/dashboard-and-insight.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/ui/dashboard-and-insight.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/ui/dashboard-and-insight.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/forms/ticket-form.md; docs/en/03-domain/service-desk/ticket/ticket-model.md</t>
+  </si>
+  <si>
+    <t>docs/en/04-client-engineering/ui/dashboard-and-insight.md; docs/en/03-domain/service-desk/ticket/ticket-history.md</t>
   </si>
 </sst>
 </file>
@@ -1732,7 +1774,7 @@
         <v>6</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>39</v>
+        <v>215</v>
       </c>
       <c r="M4" s="7" t="s">
         <v>204</v>
@@ -1937,7 +1979,7 @@
         <v>6</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>39</v>
+        <v>216</v>
       </c>
       <c r="M9" s="7" t="s">
         <v>204</v>
@@ -2388,7 +2430,7 @@
         <v>201</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>68</v>
+        <v>217</v>
       </c>
       <c r="M20" s="7" t="s">
         <v>203</v>
@@ -2429,7 +2471,7 @@
         <v>201</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>68</v>
+        <v>218</v>
       </c>
       <c r="M21" s="7" t="s">
         <v>203</v>
@@ -2470,7 +2512,7 @@
         <v>201</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>68</v>
+        <v>219</v>
       </c>
       <c r="M22" s="7" t="s">
         <v>203</v>
@@ -2511,7 +2553,7 @@
         <v>201</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>68</v>
+        <v>220</v>
       </c>
       <c r="M23" s="7" t="s">
         <v>203</v>
@@ -2634,7 +2676,7 @@
         <v>6</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>39</v>
+        <v>221</v>
       </c>
       <c r="M26" s="7" t="s">
         <v>204</v>
@@ -2839,7 +2881,7 @@
         <v>6</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>39</v>
+        <v>222</v>
       </c>
       <c r="M31" s="7" t="s">
         <v>204</v>
@@ -3290,7 +3332,7 @@
         <v>201</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>68</v>
+        <v>223</v>
       </c>
       <c r="M42" s="7" t="s">
         <v>203</v>
@@ -3331,7 +3373,7 @@
         <v>201</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>68</v>
+        <v>224</v>
       </c>
       <c r="M43" s="7" t="s">
         <v>203</v>
@@ -3372,7 +3414,7 @@
         <v>201</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>68</v>
+        <v>225</v>
       </c>
       <c r="M44" s="7" t="s">
         <v>203</v>
@@ -3413,7 +3455,7 @@
         <v>201</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>68</v>
+        <v>226</v>
       </c>
       <c r="M45" s="7" t="s">
         <v>203</v>
@@ -3861,7 +3903,7 @@
         <v>108</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>39</v>
+        <v>227</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>114</v>
@@ -3953,7 +3995,7 @@
         <v>108</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>136</v>
+        <v>228</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>137</v>

</xml_diff>